<commit_message>
chore: 更新 Test 表数据
</commit_message>
<xml_diff>
--- a/Excel/Test/Test.xlsx
+++ b/Excel/Test/Test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityWork\zhou-master\Excel\Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4542B5EE-12C4-4168-A06C-CCCDF7F389D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{850E1080-FECB-4A98-989C-9D760D1DFA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24144" windowHeight="14447" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -323,7 +323,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="617">
   <si>
     <t>Id</t>
   </si>
@@ -1577,9 +1577,6 @@
   </si>
   <si>
     <t>Normal</t>
-  </si>
-  <si>
-    <t>电大</t>
   </si>
   <si>
     <t>1,4</t>
@@ -2179,6 +2176,10 @@
   </si>
   <si>
     <t>{"Expression":"Target.MainSkill.Power = Target.MainSkill.Power - 1f / 60 * (Target.MainSkill.Power &lt; 1f / 60 ? 0 : 2)","绑定进度条":"圆"}</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>电大</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
 </sst>
@@ -2267,7 +2268,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -2287,6 +2288,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3339,7 +3343,7 @@
         <v>140</v>
       </c>
       <c r="AL5" s="5" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AM5" s="3" t="s">
         <v>142</v>
@@ -3416,7 +3420,7 @@
         <v>155</v>
       </c>
       <c r="AL6" s="5" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AM6" s="3"/>
     </row>
@@ -5069,35 +5073,38 @@
       <c r="BF6" s="1">
         <v>0.25</v>
       </c>
+      <c r="BP6" s="7" t="s">
+        <v>616</v>
+      </c>
       <c r="BQ6" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="CB6" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="CB6" s="1" t="s">
+      <c r="CH6" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="CH6" s="1" t="s">
+      <c r="CI6" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="CI6" s="1" t="s">
+      <c r="CJ6" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="CJ6" s="1" t="s">
+      <c r="CK6" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="CK6" s="1" t="s">
+      <c r="CO6" s="1" t="s">
         <v>424</v>
-      </c>
-      <c r="CO6" s="1" t="s">
-        <v>425</v>
       </c>
       <c r="CS6" s="1">
         <v>12</v>
       </c>
       <c r="CV6" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="CZ6" s="1" t="s">
         <v>426</v>
-      </c>
-      <c r="CZ6" s="1" t="s">
-        <v>427</v>
       </c>
       <c r="DE6" s="1">
         <v>1</v>
@@ -5111,19 +5118,19 @@
     </row>
     <row r="7" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="R7" s="1" t="s">
         <v>431</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>432</v>
       </c>
       <c r="AC7" s="1">
         <v>2</v>
@@ -5141,27 +5148,27 @@
         <v>99</v>
       </c>
       <c r="CI7" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="K8" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>435</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>436</v>
       </c>
       <c r="AC8" s="1">
         <v>2</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="AX8" s="1" t="s">
         <v>417</v>
@@ -5176,30 +5183,30 @@
         <v>1</v>
       </c>
       <c r="CM8" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="CZ8" s="1" t="s">
         <v>438</v>
-      </c>
-      <c r="CZ8" s="1" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="10" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="AC10" s="1">
         <v>1</v>
       </c>
       <c r="AG10" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="BD10" s="1">
         <v>1</v>
@@ -5217,21 +5224,21 @@
         <v>1</v>
       </c>
       <c r="BY10" s="6" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="CO10" s="1" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="12" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="J12" s="1" t="s">
         <v>444</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>445</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>413</v>
@@ -5267,42 +5274,42 @@
         <v>1</v>
       </c>
       <c r="BY12" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="CB12" s="1" t="s">
         <v>62</v>
       </c>
       <c r="CH12" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="CI12" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="CJ12" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="CJ12" s="1" t="s">
+      <c r="CK12" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="CK12" s="1" t="s">
+      <c r="CO12" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="CV12" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="CO12" s="1" t="s">
-        <v>432</v>
-      </c>
-      <c r="CV12" s="1" t="s">
-        <v>450</v>
-      </c>
       <c r="CZ12" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="13" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>413</v>
@@ -5311,7 +5318,7 @@
         <v>1</v>
       </c>
       <c r="AG13" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="BD13" s="1">
         <v>1</v>
@@ -5332,7 +5339,7 @@
         <v>413</v>
       </c>
       <c r="CO13" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="CP13" s="1">
         <v>200</v>
@@ -5346,13 +5353,13 @@
     </row>
     <row r="14" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>413</v>
@@ -5361,7 +5368,7 @@
         <v>1</v>
       </c>
       <c r="AG14" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="BD14" s="1">
         <v>1</v>
@@ -5379,21 +5386,21 @@
         <v>1</v>
       </c>
       <c r="BY14" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="CO14" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="CV14" s="1" t="s">
         <v>454</v>
-      </c>
-      <c r="CV14" s="1" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="16" spans="1:114" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>456</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>457</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>413</v>
@@ -5402,16 +5409,16 @@
         <v>2</v>
       </c>
       <c r="AO16" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="AR16" s="1" t="s">
         <v>458</v>
-      </c>
-      <c r="AR16" s="1" t="s">
-        <v>459</v>
       </c>
       <c r="AV16" s="1">
         <v>8</v>
       </c>
       <c r="AX16" s="1" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="AZ16" s="1">
         <v>1.5</v>
@@ -5423,10 +5430,10 @@
         <v>6</v>
       </c>
       <c r="CI16" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="CO16" s="1" t="s">
         <v>461</v>
-      </c>
-      <c r="CO16" s="1" t="s">
-        <v>462</v>
       </c>
       <c r="CP16" s="1">
         <v>-50</v>
@@ -5438,24 +5445,24 @@
         <v>3</v>
       </c>
       <c r="CV16" s="1" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="17" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="L17" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>465</v>
-      </c>
       <c r="Q17" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AC17" s="1">
         <v>2</v>
@@ -5467,15 +5474,15 @@
         <v>1</v>
       </c>
       <c r="CV17" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="18" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>413</v>
@@ -5487,7 +5494,7 @@
         <v>415</v>
       </c>
       <c r="AR18" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AV18" s="1">
         <v>3.5</v>
@@ -5505,25 +5512,25 @@
         <v>62</v>
       </c>
       <c r="CH18" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="CI18" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="CJ18" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="CO18" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="CP18" s="1">
         <v>-0.8</v>
       </c>
       <c r="CV18" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="CZ18" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="19" spans="1:113" x14ac:dyDescent="0.25">
@@ -5531,10 +5538,10 @@
         <v>160</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>413</v>
@@ -5543,7 +5550,7 @@
         <v>1</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="BD19" s="1">
         <v>1</v>
@@ -5564,7 +5571,7 @@
         <v>413</v>
       </c>
       <c r="CO19" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="CP19" s="1">
         <v>100</v>
@@ -5575,10 +5582,10 @@
     </row>
     <row r="20" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="I20" s="1">
         <v>1</v>
@@ -5593,10 +5600,10 @@
         <v>1</v>
       </c>
       <c r="AG20" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="AX20" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="AZ20" s="1">
         <v>0.05</v>
@@ -5611,7 +5618,7 @@
         <v>0.5</v>
       </c>
       <c r="CZ20" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="DE20" s="1">
         <v>1</v>
@@ -5625,16 +5632,16 @@
     </row>
     <row r="22" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>474</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="J22" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="K22" s="1" t="s">
         <v>475</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>476</v>
       </c>
       <c r="X22" s="1">
         <v>1</v>
@@ -5658,7 +5665,7 @@
         <v>413</v>
       </c>
       <c r="CV22" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="23" spans="1:113" x14ac:dyDescent="0.25">
@@ -5666,13 +5673,13 @@
         <v>170</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AC23" s="1">
         <v>7</v>
@@ -5681,7 +5688,7 @@
         <v>1</v>
       </c>
       <c r="AG23" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="AN23" s="1">
         <v>1</v>
@@ -5700,17 +5707,17 @@
       </c>
     </row>
     <row r="25" spans="1:113" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>418</v>
+      <c r="A25" s="6" t="s">
+        <v>616</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>412</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="L25" s="1" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="X25" s="1">
         <v>1</v>
@@ -5743,7 +5750,7 @@
         <v>0.04</v>
       </c>
       <c r="BP25" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="BT25" s="1">
         <v>2.5</v>
@@ -5758,48 +5765,48 @@
         <v>1</v>
       </c>
       <c r="BY25" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="CB25" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="CB25" s="1" t="s">
+      <c r="CF25" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="CG25" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="CH25" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="CI25" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="CF25" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="CG25" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="CH25" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="CI25" s="1" t="s">
+      <c r="CJ25" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="CJ25" s="1" t="s">
+      <c r="CK25" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="CV25" s="1" t="s">
         <v>483</v>
-      </c>
-      <c r="CK25" s="1" t="s">
-        <v>449</v>
-      </c>
-      <c r="CV25" s="1" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="26" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AC26" s="1">
         <v>1</v>
       </c>
       <c r="AG26" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="BD26" s="1">
         <v>1</v>
@@ -5816,13 +5823,13 @@
         <v>142</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="O28" s="1" t="s">
         <v>414</v>
@@ -5831,7 +5838,7 @@
         <v>1</v>
       </c>
       <c r="AG28" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="BT28" s="1">
         <v>2.5</v>
@@ -5851,89 +5858,89 @@
     </row>
     <row r="31" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="K31" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="L31" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="L31" s="1" t="s">
+      <c r="AC31" s="1">
+        <v>1</v>
+      </c>
+      <c r="AF31" s="1">
+        <v>1</v>
+      </c>
+      <c r="AG31" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="BD31" s="1">
+        <v>1</v>
+      </c>
+      <c r="CV31" s="1" t="s">
         <v>487</v>
-      </c>
-      <c r="AC31" s="1">
-        <v>1</v>
-      </c>
-      <c r="AF31" s="1">
-        <v>1</v>
-      </c>
-      <c r="AG31" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="BD31" s="1">
-        <v>1</v>
-      </c>
-      <c r="CV31" s="1" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="32" spans="1:113" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="AC32" s="1">
+        <v>1</v>
+      </c>
+      <c r="AF32" s="1">
+        <v>1</v>
+      </c>
+      <c r="AG32" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="BD32" s="1">
+        <v>1</v>
+      </c>
+      <c r="CV32" s="1" t="s">
         <v>489</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="AC32" s="1">
-        <v>1</v>
-      </c>
-      <c r="AF32" s="1">
-        <v>1</v>
-      </c>
-      <c r="AG32" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="BD32" s="1">
-        <v>1</v>
-      </c>
-      <c r="CV32" s="1" t="s">
-        <v>490</v>
       </c>
     </row>
     <row r="33" spans="1:100" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="AC33" s="1">
+        <v>1</v>
+      </c>
+      <c r="AF33" s="1">
+        <v>1</v>
+      </c>
+      <c r="AG33" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="BD33" s="1">
+        <v>1</v>
+      </c>
+      <c r="CV33" s="1" t="s">
         <v>491</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>486</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>487</v>
-      </c>
-      <c r="AC33" s="1">
-        <v>1</v>
-      </c>
-      <c r="AF33" s="1">
-        <v>1</v>
-      </c>
-      <c r="AG33" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="BD33" s="1">
-        <v>1</v>
-      </c>
-      <c r="CV33" s="1" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="684" spans="91:91" x14ac:dyDescent="0.25">
@@ -5996,7 +6003,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.05" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
@@ -6019,37 +6026,37 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>496</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>502</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -6063,40 +6070,40 @@
         <v>84</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>504</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>509</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>510</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>58</v>
       </c>
       <c r="M2" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>511</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="O2" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>513</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>514</v>
       </c>
       <c r="Q2" s="1" t="s">
         <v>379</v>
@@ -6154,55 +6161,55 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="K4" s="1">
         <v>5</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>517</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="K6" s="1">
         <v>99999</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>521</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>522</v>
       </c>
       <c r="K7" s="1">
         <v>12</v>
@@ -6210,69 +6217,69 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>522</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>523</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="J8" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="J8" s="3" t="s">
+      <c r="Q8" s="3" t="s">
         <v>525</v>
-      </c>
-      <c r="Q8" s="3" t="s">
-        <v>526</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>527</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>529</v>
-      </c>
       <c r="Q10" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="K11" s="1">
         <v>0.8</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="J12" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="Q12" s="3" t="s">
         <v>533</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>534</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
@@ -6280,10 +6287,10 @@
         <v>165</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="Q14" s="3" t="s">
         <v>535</v>
-      </c>
-      <c r="Q14" s="3" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
@@ -6291,10 +6298,15 @@
         <v>414</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
+      </c>
+    </row>
+    <row r="18" spans="10:10" x14ac:dyDescent="0.25">
+      <c r="J18" s="3" t="s">
+        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -6320,7 +6332,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -6331,7 +6343,7 @@
         <v>52</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>379</v>
@@ -6353,16 +6365,16 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>540</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>541</v>
       </c>
     </row>
   </sheetData>
@@ -6402,19 +6414,19 @@
         <v>54</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>77</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>544</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>545</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>368</v>
@@ -6457,64 +6469,64 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>546</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>547</v>
       </c>
       <c r="E4" s="1">
         <v>4</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>550</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>551</v>
       </c>
       <c r="E5" s="1">
         <v>10</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>553</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>554</v>
       </c>
       <c r="E6" s="1">
         <v>10</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="E7" s="1">
         <v>2.25</v>
@@ -6523,18 +6535,18 @@
         <v>2</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="E8" s="1">
         <v>3</v>
@@ -6543,12 +6555,12 @@
         <v>2</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C12" s="1" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>
@@ -6576,34 +6588,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>561</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>563</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>564</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>569</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>570</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -6611,34 +6623,34 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>571</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>574</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>576</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>579</v>
-      </c>
       <c r="K2" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>104</v>
@@ -6687,10 +6699,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="K5" s="1">
         <v>60</v>
@@ -6701,10 +6713,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>581</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>582</v>
       </c>
       <c r="K7" s="1">
         <v>60</v>
@@ -6744,22 +6756,22 @@
         <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>583</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>584</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>86</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>316</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>59</v>
@@ -6788,7 +6800,7 @@
         <v>128</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>128</v>
@@ -6824,28 +6836,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>587</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>588</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>589</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>593</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>594</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -6853,28 +6865,28 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>599</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>601</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>602</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>603</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -6908,28 +6920,28 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>604</v>
       </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>605</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>606</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>607</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>608</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>609</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>610</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: 补充 SpineBoneDump.meta 与 Excel 表更新
</commit_message>
<xml_diff>
--- a/Excel/Test/Test.xlsx
+++ b/Excel/Test/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UnityWork\zhou-master\Excel\Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469F9B7B-E1DD-4EE8-8D46-9073ABAD34A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02739AC-462A-4AAA-A63F-92411464B789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24144" windowHeight="14447" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -323,7 +323,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="621">
   <si>
     <t>Id</t>
   </si>
@@ -2191,6 +2191,10 @@
   </si>
   <si>
     <t>myrtle_attack_01_start_taiko#1</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>agoat2_skill_03_buff_01</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
 </sst>
@@ -6580,7 +6584,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.05" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.25" style="1" customWidth="1"/>
@@ -6709,8 +6713,8 @@
       <c r="A5" s="3" t="s">
         <v>524</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>619</v>
+      <c r="B5" s="5" t="s">
+        <v>620</v>
       </c>
       <c r="K5" s="1">
         <v>60</v>
@@ -6738,6 +6742,11 @@
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
         <v>618</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>619</v>
       </c>
     </row>
   </sheetData>

</xml_diff>